<commit_message>
bug: fixed R10 path issue
</commit_message>
<xml_diff>
--- a/templates/PipelineWorksheetMASTER.xlsx
+++ b/templates/PipelineWorksheetMASTER.xlsx
@@ -1,26 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\projects\alindsay\Projects\ngs-pipeline-launcher\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\apps\production\ngs-pipeline-launcher\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF644AE3-A322-4961-97B8-5AAB3FDFA9F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{274A9499-78AF-4A0B-9CCF-FE33650D4D1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="24540" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1770" yWindow="1770" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PipelineWorksheet" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="146">
   <si>
     <t>[Header]</t>
   </si>
@@ -61,9 +74,6 @@
     <t>[Pipelines]</t>
   </si>
   <si>
-    <t>/nfs/APL_Genomics/apps/production/covid/pl_ncov_auto_V7.py</t>
-  </si>
-  <si>
     <t>Barcode</t>
   </si>
   <si>
@@ -418,9 +428,6 @@
     <t># e.g., 230711_N_I_063</t>
   </si>
   <si>
-    <t># e.g., /nfs/APL_Genomics/230711_N_I_063/</t>
-  </si>
-  <si>
     <t>/nfs/APL_Genomics/apps/production/influenza/flu.sh</t>
   </si>
   <si>
@@ -452,6 +459,18 @@
   </si>
   <si>
     <t>[Samples]</t>
+  </si>
+  <si>
+    <t>/nfs/APL_Genomics/apps/production/covid/pl_ncov_auto_V8.py</t>
+  </si>
+  <si>
+    <t># e.g., /nfs/APL_Genomics/raw/ncov-raw/2026/YOUR_RUN/</t>
+  </si>
+  <si>
+    <t>ncov-R10</t>
+  </si>
+  <si>
+    <t>/nfs/APL_Genomics/apps/production/covid/ncov-R10.sh</t>
   </si>
 </sst>
 </file>
@@ -1178,7 +1197,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1248,16 +1267,6 @@
     <xf numFmtId="0" fontId="0" fillId="40" borderId="25" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="40" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="40" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="37" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="39" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="40" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1587,7 +1596,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F226"/>
+  <dimension ref="A1:F228"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.140625" customWidth="1"/>
@@ -1608,7 +1617,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1616,7 +1625,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1655,7 +1664,7 @@
         <v>10</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D8" s="15"/>
     </row>
@@ -1664,1759 +1673,1777 @@
         <v>11</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D9" s="16"/>
     </row>
     <row r="10" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>18</v>
+        <v>144</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="D10" s="16"/>
     </row>
     <row r="11" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D11" s="16"/>
     </row>
     <row r="12" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D12" s="16"/>
     </row>
     <row r="13" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D13" s="16"/>
     </row>
     <row r="14" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D14" s="16"/>
     </row>
     <row r="15" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D15" s="16"/>
     </row>
     <row r="16" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" s="16"/>
+    </row>
+    <row r="17" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B17" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="D16" s="16"/>
-    </row>
-    <row r="17" spans="1:4" s="37" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="35" t="s">
-        <v>140</v>
-      </c>
-      <c r="D17" s="39"/>
-    </row>
-    <row r="18" spans="1:4" s="37" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="35" t="s">
-        <v>134</v>
-      </c>
-      <c r="B18" s="37" t="s">
-        <v>141</v>
-      </c>
-      <c r="D18" s="39"/>
-    </row>
-    <row r="19" spans="1:4" s="23" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="D19" s="24"/>
-    </row>
-    <row r="20" spans="1:4" s="19" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="19" t="s">
+      <c r="D17" s="16"/>
+    </row>
+    <row r="18" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="D18" s="16"/>
+    </row>
+    <row r="19" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="D19" s="16"/>
+    </row>
+    <row r="20" spans="1:4" s="23" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D20" s="24"/>
+    </row>
+    <row r="21" spans="1:4" s="19" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="D20" s="20"/>
-    </row>
-    <row r="21" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="8" t="s">
+      <c r="D21" s="20"/>
+    </row>
+    <row r="22" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B21" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D21" s="17"/>
-    </row>
-    <row r="22" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B22" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="D22" s="18"/>
+      <c r="B22" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="D22" s="17"/>
     </row>
     <row r="23" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="D23" s="18"/>
     </row>
     <row r="24" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
-        <v>20</v>
+        <v>144</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="D24" s="18"/>
     </row>
     <row r="25" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>17</v>
+        <v>131</v>
       </c>
       <c r="D25" s="18"/>
     </row>
     <row r="26" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="D26" s="18"/>
     </row>
     <row r="27" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D27" s="18"/>
     </row>
     <row r="28" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="B28" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="D28" s="18"/>
+    </row>
+    <row r="29" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D29" s="18"/>
+    </row>
+    <row r="30" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="D30" s="18"/>
+    </row>
+    <row r="31" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D31" s="18"/>
+    </row>
+    <row r="32" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="D28" s="18"/>
-    </row>
-    <row r="29" spans="1:4" s="38" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="36" t="s">
-        <v>30</v>
-      </c>
-      <c r="B29" s="38" t="s">
-        <v>17</v>
-      </c>
-      <c r="D29" s="40"/>
-    </row>
-    <row r="30" spans="1:4" s="38" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="36" t="s">
+      <c r="B32" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="B30" s="38" t="s">
-        <v>142</v>
-      </c>
-      <c r="D30" s="40"/>
-    </row>
-    <row r="31" spans="1:4" s="38" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="36" t="s">
+      <c r="D32" s="18"/>
+    </row>
+    <row r="33" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D33" s="18"/>
+    </row>
+    <row r="34" spans="1:6" s="30" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D34" s="31"/>
+    </row>
+    <row r="35" spans="1:6" s="33" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="32" t="s">
+        <v>141</v>
+      </c>
+      <c r="D35" s="34"/>
+    </row>
+    <row r="36" spans="1:6" s="36" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="B36" s="36" t="s">
+        <v>129</v>
+      </c>
+      <c r="C36" s="36" t="s">
+        <v>14</v>
+      </c>
+      <c r="D36" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="E36" s="36" t="s">
+        <v>133</v>
+      </c>
+      <c r="F36" s="36" t="s">
         <v>134</v>
       </c>
-      <c r="B31" s="38" t="s">
-        <v>139</v>
-      </c>
-      <c r="D31" s="40"/>
-    </row>
-    <row r="32" spans="1:4" s="30" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="D32" s="31"/>
-    </row>
-    <row r="33" spans="1:6" s="33" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="32" t="s">
-        <v>143</v>
-      </c>
-      <c r="D33" s="34"/>
-    </row>
-    <row r="34" spans="1:6" s="42" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="41" t="s">
-        <v>14</v>
-      </c>
-      <c r="B34" s="42" t="s">
-        <v>130</v>
-      </c>
-      <c r="C34" s="42" t="s">
-        <v>15</v>
-      </c>
-      <c r="D34" s="42" t="s">
-        <v>16</v>
-      </c>
-      <c r="E34" s="42" t="s">
-        <v>135</v>
-      </c>
-      <c r="F34" s="42" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" s="26" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="25">
+    </row>
+    <row r="37" spans="1:6" s="26" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="25">
         <v>1</v>
       </c>
-      <c r="B35" s="26" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" s="28" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="27">
-        <v>2</v>
-      </c>
-      <c r="B36" s="28" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" s="28" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="27">
-        <v>3</v>
-      </c>
-      <c r="B37" s="28" t="s">
-        <v>36</v>
+      <c r="B37" s="26" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="38" spans="1:6" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="27">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B38" s="28" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="39" spans="1:6" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="27">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B39" s="28" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="40" spans="1:6" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="27">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B40" s="28" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="41" spans="1:6" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="27">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B41" s="28" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="42" spans="1:6" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="27">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B42" s="28" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="43" spans="1:6" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="27">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B43" s="28" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="44" spans="1:6" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="27">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B44" s="28" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="45" spans="1:6" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="27">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B45" s="28" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="46" spans="1:6" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="27">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B46" s="28" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="47" spans="1:6" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="27">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B47" s="28" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="48" spans="1:6" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="27">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B48" s="28" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="49" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="27">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B49" s="28" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="50" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="27">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B50" s="28" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="51" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="27">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B51" s="28" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="52" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="27">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B52" s="28" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="53" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="27">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B53" s="28" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="54" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="27">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B54" s="28" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="55" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="27">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B55" s="28" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="56" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="27">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B56" s="28" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="57" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="27">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B57" s="28" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="58" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="27">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B58" s="28" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="59" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="27">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B59" s="28" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="60" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="27">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B60" s="28" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="61" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="27">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B61" s="28" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="62" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="27">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B62" s="28" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="63" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="27">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B63" s="28" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="64" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="27">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B64" s="28" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="65" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="27">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B65" s="28" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="66" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="27">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B66" s="28" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="67" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="27">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B67" s="28" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="68" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="27">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B68" s="28" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="69" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="27">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B69" s="28" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="70" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="27">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B70" s="28" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="71" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="27">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B71" s="28" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="72" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="27">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B72" s="28" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="73" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="27">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B73" s="28" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="74" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="27">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B74" s="28" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="75" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="27">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B75" s="28" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="76" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="27">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B76" s="28" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="77" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="27">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B77" s="28" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="78" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="27">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B78" s="28" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="79" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="27">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B79" s="28" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="80" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="27">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B80" s="28" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="81" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="27">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B81" s="28" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="82" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="27">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B82" s="28" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="83" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="27">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B83" s="28" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="84" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="27">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B84" s="28" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="85" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="27">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B85" s="28" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="86" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="27">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B86" s="28" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="87" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="27">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B87" s="28" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="88" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="27">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B88" s="28" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="89" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="27">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B89" s="28" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="90" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="27">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B90" s="28" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="91" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="27">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B91" s="28" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="92" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="27">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B92" s="28" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="93" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="27">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B93" s="28" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="94" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="27">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B94" s="28" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="95" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="27">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B95" s="28" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="96" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="27">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B96" s="28" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="97" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="27">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B97" s="28" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="98" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="27">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B98" s="28" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="99" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="27">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B99" s="28" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="100" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="27">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B100" s="28" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="101" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="27">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B101" s="28" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="102" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="27">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B102" s="28" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="103" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="27">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B103" s="28" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="104" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="27">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B104" s="28" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="105" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="27">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B105" s="28" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="106" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="27">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B106" s="28" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="107" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="27">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B107" s="28" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="108" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="27">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B108" s="28" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="109" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="27">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B109" s="28" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="110" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="27">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B110" s="28" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
     </row>
     <row r="111" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="27">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B111" s="28" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="112" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="27">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B112" s="28" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="113" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="27">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B113" s="28" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="114" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="27">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B114" s="28" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="115" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="27">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B115" s="28" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="116" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="27">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B116" s="28" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="117" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="27">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B117" s="28" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="118" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="27">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B118" s="28" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="119" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="27">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B119" s="28" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="120" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="27">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B120" s="28" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="121" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="27">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B121" s="28" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="122" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="27">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B122" s="28" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="123" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="27">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B123" s="28" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="124" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="27">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B124" s="28" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="125" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="27">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B125" s="28" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="126" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="27">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B126" s="28" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="127" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="27">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B127" s="28" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="128" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="27">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B128" s="28" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="129" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="27">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B129" s="28" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="130" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A130" s="28">
-        <v>96</v>
+      <c r="A130" s="27">
+        <v>94</v>
       </c>
       <c r="B130" s="28" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="131" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="27">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B131" s="28" t="s">
-        <v>34</v>
+        <v>127</v>
       </c>
     </row>
     <row r="132" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="28">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B132" s="28" t="s">
-        <v>35</v>
+        <v>128</v>
       </c>
     </row>
     <row r="133" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="27">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B133" s="28" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="134" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="28">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B134" s="28" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="135" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="27">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B135" s="28" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="136" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A136" s="28">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B136" s="28" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="137" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A137" s="27">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B137" s="28" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="138" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A138" s="28">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B138" s="28" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="139" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A139" s="27">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B139" s="28" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="140" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A140" s="28">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B140" s="28" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="141" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A141" s="27">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B141" s="28" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="142" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A142" s="28">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B142" s="28" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="143" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A143" s="27">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B143" s="28" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="144" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A144" s="28">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B144" s="28" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="145" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A145" s="27">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B145" s="28" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="146" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A146" s="28">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B146" s="28" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="147" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A147" s="27">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B147" s="28" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="148" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A148" s="28">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B148" s="28" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="149" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A149" s="27">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B149" s="28" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="150" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A150" s="28">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B150" s="28" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="151" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A151" s="27">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B151" s="28" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="152" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A152" s="28">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B152" s="28" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="153" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A153" s="27">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B153" s="28" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="154" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A154" s="28">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B154" s="28" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="155" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A155" s="27">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B155" s="28" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="156" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A156" s="28">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B156" s="28" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="157" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A157" s="27">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B157" s="28" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="158" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A158" s="28">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B158" s="28" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="159" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A159" s="27">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B159" s="28" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="160" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A160" s="28">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B160" s="28" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="161" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A161" s="27">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B161" s="28" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="162" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A162" s="28">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B162" s="28" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="163" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A163" s="27">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B163" s="28" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="164" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A164" s="28">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B164" s="28" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="165" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A165" s="27">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B165" s="28" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="166" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A166" s="28">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B166" s="28" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="167" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A167" s="27">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B167" s="28" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="168" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A168" s="28">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B168" s="28" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="169" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A169" s="27">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B169" s="28" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="170" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A170" s="28">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B170" s="28" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="171" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A171" s="27">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B171" s="28" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="172" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A172" s="28">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B172" s="28" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="173" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A173" s="27">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B173" s="28" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="174" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A174" s="28">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B174" s="28" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="175" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A175" s="27">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B175" s="28" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="176" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A176" s="28">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B176" s="28" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="177" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A177" s="27">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B177" s="28" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="178" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A178" s="28">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B178" s="28" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="179" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A179" s="27">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B179" s="28" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="180" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A180" s="28">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B180" s="28" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="181" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A181" s="27">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B181" s="28" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="182" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A182" s="28">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B182" s="28" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="183" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A183" s="27">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B183" s="28" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="184" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A184" s="28">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B184" s="28" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="185" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A185" s="27">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B185" s="28" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="186" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A186" s="28">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B186" s="28" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="187" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A187" s="27">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B187" s="28" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="188" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A188" s="28">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B188" s="28" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="189" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A189" s="27">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B189" s="28" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="190" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A190" s="28">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B190" s="28" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="191" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A191" s="27">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B191" s="28" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="192" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A192" s="28">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B192" s="28" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="193" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A193" s="27">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B193" s="28" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="194" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A194" s="28">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B194" s="28" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="195" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A195" s="27">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B195" s="28" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="196" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A196" s="28">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B196" s="28" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="197" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A197" s="27">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B197" s="28" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="198" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A198" s="28">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B198" s="28" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="199" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A199" s="27">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B199" s="28" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="200" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A200" s="28">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B200" s="28" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="201" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A201" s="27">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B201" s="28" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="202" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A202" s="28">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B202" s="28" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="203" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A203" s="27">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B203" s="28" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="204" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A204" s="28">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B204" s="28" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="205" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A205" s="27">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B205" s="28" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="206" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A206" s="28">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B206" s="28" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
     </row>
     <row r="207" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A207" s="27">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B207" s="28" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="208" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A208" s="28">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B208" s="28" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="209" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A209" s="27">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B209" s="28" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="210" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A210" s="28">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B210" s="28" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="211" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A211" s="27">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B211" s="28" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="212" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A212" s="28">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B212" s="28" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="213" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A213" s="27">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B213" s="28" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="214" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A214" s="28">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B214" s="28" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="215" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A215" s="27">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B215" s="28" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="216" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A216" s="28">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B216" s="28" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="217" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A217" s="27">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B217" s="28" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="218" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A218" s="28">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B218" s="28" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="219" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A219" s="27">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B219" s="28" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="220" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A220" s="28">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B220" s="28" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="221" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A221" s="27">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B221" s="28" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="222" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A222" s="28">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B222" s="28" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="223" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A223" s="27">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B223" s="28" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="224" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A224" s="28">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B224" s="28" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="225" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A225" s="27">
+        <v>189</v>
+      </c>
+      <c r="B225" s="28" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A226" s="28">
+        <v>190</v>
+      </c>
+      <c r="B226" s="28" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="227" spans="1:2" s="28" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A227" s="27">
         <v>191</v>
       </c>
-      <c r="B225" s="28" t="s">
+      <c r="B227" s="28" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2" s="29" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A228" s="29">
+        <v>192</v>
+      </c>
+      <c r="B228" s="29" t="s">
         <v>128</v>
-      </c>
-    </row>
-    <row r="226" spans="1:2" s="29" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A226" s="29">
-        <v>192</v>
-      </c>
-      <c r="B226" s="29" t="s">
-        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: update master worksheet
</commit_message>
<xml_diff>
--- a/templates/PipelineWorksheetMASTER.xlsx
+++ b/templates/PipelineWorksheetMASTER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\projects\alindsay\Projects\ngs-pipeline-launcher\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1721CD42-4000-4CD3-BED2-2F1BA2AA57C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8410514B-0078-44A1-ACF7-0B8BA1E0B785}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="1410" windowWidth="27435" windowHeight="19470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1125" yWindow="1125" windowWidth="27435" windowHeight="19470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PipelineWorksheet" sheetId="1" r:id="rId1"/>
@@ -1072,7 +1072,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1096,36 +1096,32 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="40" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="40" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="39" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="39" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="39" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="39" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1459,39 +1455,36 @@
     <col min="5" max="18" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="19" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
+    <row r="1" spans="1:4" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="20"/>
+      <c r="D1" s="18"/>
     </row>
     <row r="2" spans="1:4" s="15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="16" t="s">
+      <c r="C2" s="16" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:4" s="15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="C3" s="16" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="4" spans="1:4" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="D4" s="18"/>
-    </row>
-    <row r="5" spans="1:4" s="21" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="21" t="s">
+    <row r="5" spans="1:4" s="19" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="22"/>
+      <c r="D5" s="20"/>
     </row>
     <row r="6" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="19" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="13" t="s">
@@ -1500,7 +1493,7 @@
       <c r="D6" s="14"/>
     </row>
     <row r="7" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="19" t="s">
         <v>5</v>
       </c>
       <c r="B7" s="13" t="s">
@@ -1509,7 +1502,7 @@
       <c r="D7" s="14"/>
     </row>
     <row r="8" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="19" t="s">
         <v>138</v>
       </c>
       <c r="B8" s="13" t="s">
@@ -1518,7 +1511,7 @@
       <c r="D8" s="14"/>
     </row>
     <row r="9" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="19" t="s">
         <v>11</v>
       </c>
       <c r="B9" s="13" t="s">
@@ -1527,7 +1520,7 @@
       <c r="D9" s="14"/>
     </row>
     <row r="10" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="19" t="s">
         <v>13</v>
       </c>
       <c r="B10" s="13" t="s">
@@ -1536,7 +1529,7 @@
       <c r="D10" s="14"/>
     </row>
     <row r="11" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="21" t="s">
+      <c r="A11" s="19" t="s">
         <v>15</v>
       </c>
       <c r="B11" s="13" t="s">
@@ -1545,7 +1538,7 @@
       <c r="D11" s="14"/>
     </row>
     <row r="12" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="19" t="s">
         <v>17</v>
       </c>
       <c r="B12" s="13" t="s">
@@ -1554,7 +1547,7 @@
       <c r="D12" s="14"/>
     </row>
     <row r="13" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="19" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="13" t="s">
@@ -1563,7 +1556,7 @@
       <c r="D13" s="14"/>
     </row>
     <row r="14" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="21" t="s">
+      <c r="A14" s="19" t="s">
         <v>21</v>
       </c>
       <c r="B14" s="13" t="s">
@@ -1572,7 +1565,7 @@
       <c r="D14" s="14"/>
     </row>
     <row r="15" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="21" t="s">
+      <c r="A15" s="19" t="s">
         <v>23</v>
       </c>
       <c r="B15" s="13" t="s">
@@ -1581,13 +1574,13 @@
       <c r="D15" s="14"/>
     </row>
     <row r="16" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="21" t="s">
+      <c r="A16" s="19" t="s">
         <v>132</v>
       </c>
       <c r="D16" s="14"/>
     </row>
     <row r="17" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="21" t="s">
+      <c r="A17" s="19" t="s">
         <v>126</v>
       </c>
       <c r="B17" s="13" t="s">
@@ -1595,17 +1588,14 @@
       </c>
       <c r="D17" s="14"/>
     </row>
-    <row r="18" spans="1:4" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="D18" s="18"/>
-    </row>
-    <row r="19" spans="1:4" s="23" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="23" t="s">
+    <row r="19" spans="1:4" s="21" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="D19" s="24"/>
+      <c r="D19" s="22"/>
     </row>
     <row r="20" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="23" t="s">
+      <c r="A20" s="21" t="s">
         <v>4</v>
       </c>
       <c r="B20" s="11" t="s">
@@ -1614,7 +1604,7 @@
       <c r="D20" s="12"/>
     </row>
     <row r="21" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="23" t="s">
+      <c r="A21" s="21" t="s">
         <v>5</v>
       </c>
       <c r="B21" s="11" t="s">
@@ -1623,7 +1613,7 @@
       <c r="D21" s="12"/>
     </row>
     <row r="22" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="23" t="s">
+      <c r="A22" s="21" t="s">
         <v>138</v>
       </c>
       <c r="B22" s="11" t="s">
@@ -1632,7 +1622,7 @@
       <c r="D22" s="12"/>
     </row>
     <row r="23" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="23" t="s">
+      <c r="A23" s="21" t="s">
         <v>11</v>
       </c>
       <c r="B23" s="11" t="s">
@@ -1641,7 +1631,7 @@
       <c r="D23" s="12"/>
     </row>
     <row r="24" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="23" t="s">
+      <c r="A24" s="21" t="s">
         <v>13</v>
       </c>
       <c r="B24" s="11" t="s">
@@ -1650,7 +1640,7 @@
       <c r="D24" s="12"/>
     </row>
     <row r="25" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="23" t="s">
+      <c r="A25" s="21" t="s">
         <v>15</v>
       </c>
       <c r="B25" s="11" t="s">
@@ -1659,7 +1649,7 @@
       <c r="D25" s="12"/>
     </row>
     <row r="26" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="23" t="s">
+      <c r="A26" s="21" t="s">
         <v>17</v>
       </c>
       <c r="B26" s="11" t="s">
@@ -1668,7 +1658,7 @@
       <c r="D26" s="12"/>
     </row>
     <row r="27" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="23" t="s">
+      <c r="A27" s="21" t="s">
         <v>19</v>
       </c>
       <c r="B27" s="11" t="s">
@@ -1677,7 +1667,7 @@
       <c r="D27" s="12"/>
     </row>
     <row r="28" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="23" t="s">
+      <c r="A28" s="21" t="s">
         <v>21</v>
       </c>
       <c r="B28" s="11" t="s">
@@ -1686,7 +1676,7 @@
       <c r="D28" s="12"/>
     </row>
     <row r="29" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="23" t="s">
+      <c r="A29" s="21" t="s">
         <v>23</v>
       </c>
       <c r="B29" s="11" t="s">
@@ -1695,7 +1685,7 @@
       <c r="D29" s="12"/>
     </row>
     <row r="30" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="23" t="s">
+      <c r="A30" s="21" t="s">
         <v>132</v>
       </c>
       <c r="B30" s="11" t="s">
@@ -1704,16 +1694,13 @@
       <c r="D30" s="12"/>
     </row>
     <row r="31" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="23" t="s">
+      <c r="A31" s="21" t="s">
         <v>126</v>
       </c>
       <c r="B31" s="11" t="s">
         <v>131</v>
       </c>
       <c r="D31" s="12"/>
-    </row>
-    <row r="32" spans="1:4" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="D32" s="18"/>
     </row>
     <row r="33" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">

</xml_diff>